<commit_message>
docs(hubspot): atualiza Excel (schema real da consolidada, multi-cliente, correções)
- Separa vw_hubspot_leads_stages (event_date) de vw_ads_crm_results (data,
  custo FLOAT64, account_id multi-cliente, colunas extras) na aba de schema.
- Nova aba "Estado & Correções": volume real (18,7k contacts/17k deals),
  amount corrigido (R$639,3mi), MQL/SQL/Opp, associação 98% ausente (dado de
  origem), acesso Drive pendente p/ consolidada, Meta join pendente na origem.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pm33C42vpr1NbQYBizYHNb
</commit_message>
<xml_diff>
--- a/hubspot/DOC_HubSpot_BigQuery.xlsx
+++ b/hubspot/DOC_HubSpot_BigQuery.xlsx
@@ -14,6 +14,7 @@
     <sheet name="5. Schema (Tabelas)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6. Fluxo de Ingestão" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="7. Campanha &amp; Join Ads" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="8. Estado &amp; Correções" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1381,7 +1382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1426,10 +1427,10 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_hubspot_leads_stages (HubSpot, nativa)</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1444,14 +1445,14 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Dia do evento (base da série temporal).</t>
+          <t>Dia do evento (nome da coluna NESTA view HubSpot).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_hubspot_leads_stages (HubSpot, nativa)</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1473,7 +1474,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_hubspot_leads_stages (HubSpot, nativa)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1488,19 +1489,19 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Nome da campanha (Paid Social) OU ID da campanha de Ads (Paid Search).</t>
+          <t>Nome (Paid Social) OU ID da campanha de Ads (Paid Search).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_hubspot_leads_stages (HubSpot, nativa)</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>custo / impressoes / cliques</t>
+          <t>custo / impressoes / cliques / resultados / cadastros / visitas</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -1510,19 +1511,19 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Mídia — preenchido pelo ramo Ads (0 no HubSpot).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
+          <t>Sempre 0 no HubSpot (colunas de mídia; preenchidas pelo ramo Ads na consolidada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_hubspot_leads_stages (HubSpot, nativa)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>contacts</t>
+          <t>contacts / leads / lifecycle_stage_mql / lifecycle_stage_sql / opportunities</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1532,19 +1533,19 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Contatos criados no dia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
+          <t>Funil de contatos por dia (SQL/Opp ~0 na Benner: não usam esses estágios).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_hubspot_leads_stages (HubSpot, nativa)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>leads</t>
+          <t>deals_created / deals_closed / deals_lost / deals_won / clients</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1554,19 +1555,19 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Entraram no estágio Lead.</t>
+          <t>Funil de negócios / clientes por dia.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_hubspot_leads_stages (HubSpot, nativa)</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>lifecycle_stage_mql</t>
+          <t>deals_moved_any_stage</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1576,173 +1577,173 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Entraram em MQL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
+          <t>Objetos distintos com evento no dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_hubspot_leads_stages (HubSpot, nativa)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>lifecycle_stage_sql</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>INT64</t>
+          <t>NUMERIC</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Entraram em SQL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
+          <t>Valor ganho (BRL) — somado no evento deal_won (corrigido jul/2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>opportunities</t>
+          <t>account_id / account_name</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>INT64</t>
+          <t>STRING</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Entraram em Oportunidade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
+          <t>⚠️ MULTI-CLIENTE: a view tem VÁRIOS clientes. O dashboard TEM que filtrar por conta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>deals_created</t>
+          <t>data</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>INT64</t>
+          <t>DATE</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Negócios criados.</t>
+          <t>Dia do evento (NA CONSOLIDADA a coluna se chama 'data', não 'event_date').</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>deals_won / deals_lost / deals_closed</t>
+          <t>mes / semana</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>INT64</t>
+          <t>DATE / INT64</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Negócios ganhos / perdidos / fechados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
+          <t>Mês (DATE_TRUNC) e semana ISO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>clients</t>
+          <t>origem / campanha</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>INT64</t>
+          <t>STRING</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Viraram Cliente (Customer).</t>
+          <t>Mesmas dimensões; comparáveis entre Ads, RD e HubSpot.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>custo</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>NUMERIC</t>
+          <t>FLOAT64</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Valor ganho (BRL).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
+          <t>⚠️ FLOAT64 na consolidada (não INT64).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_leads_stages / vw_ads_crm_results</t>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>source_table</t>
+          <t>impressoes / cliques / resultados / cadastros / visitas</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>STRING</t>
+          <t>INT64</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Só na consolidada: 'ads' | 'rd' | 'hubspot'.</t>
+          <t>Métricas de mídia (ramo Ads).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_contacts_lifecycle</t>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Contact_ID</t>
+          <t>UTM_Campaign / UTM_Medium / UTM_Source</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1752,19 +1753,19 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Chave do contato.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
+          <t>UTMs (ramos Ads/RD; NULL no HubSpot).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_contacts_lifecycle</t>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Contact_Email / Contact_Name</t>
+          <t>grupo_anuncio / pipeline_name / Deal_Source / Deal_Lost_Reason</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -1774,51 +1775,51 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Identificação.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
+          <t>Colunas extras herdadas do esquema Ads/RD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_contacts_lifecycle</t>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Contact_Lifecycle_Stage</t>
+          <t>contacts..clients / deals_moved_any_stage / amount</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
+          <t>INT64/NUMERIC</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo funil da agregada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>vw_ads_crm_results (CONSOLIDADA / final)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
           <t>STRING</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Estágio atual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>vw_hubspot_contacts_lifecycle</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Contact_Created_At</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Criação (entrada no topo).</t>
+          <t>'ads' | 'rd' | 'hubspot' — filtre por aqui para isolar a fonte.</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1831,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Origem</t>
+          <t>Contact_ID</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1840,7 +1841,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Canal normalizado.</t>
+          <t>Chave do contato.</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1853,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Campaign_ID</t>
+          <t>Contact_Email / Contact_Name</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -1862,7 +1863,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>ID da campanha de Ads (join com Ads).</t>
+          <t>Identificação.</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1875,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Campaign_Name</t>
+          <t>Contact_Lifecycle_Stage</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1884,7 +1885,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Nome legível (Paid Social).</t>
+          <t>Estágio atual.</t>
         </is>
       </c>
     </row>
@@ -1896,51 +1897,51 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Campanha</t>
+          <t>Contact_Created_At</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Criação (entrada no topo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>vw_hubspot_contacts_lifecycle</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
           <t>STRING</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>COALESCE(nome, ID).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>vw_hubspot_contacts_lifecycle</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Became_Lead/MQL/SQL/Opportunity/Customer_Date</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Data de entrada em cada estágio (modelo v2).</t>
+          <t>Canal normalizado.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_deals_stage</t>
+          <t>vw_hubspot_contacts_lifecycle</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Deal_ID</t>
+          <t>Campaign_ID</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -1950,63 +1951,63 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Chave do negócio.</t>
+          <t>ID da campanha de Ads (join com Ads).</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_deals_stage</t>
+          <t>vw_hubspot_contacts_lifecycle</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Deal_Status / Deal_Win</t>
+          <t>Campaign_Name</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>STRING/BOOL</t>
+          <t>STRING</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>open|won|lost / ganho.</t>
+          <t>Nome legível (Paid Social).</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>vw_hubspot_deals_stage</t>
+          <t>vw_hubspot_contacts_lifecycle</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Deal_Amount / Deal_Currency</t>
+          <t>Campanha</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>NUMERIC/STRING</t>
+          <t>STRING</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Valor e moeda (BRL).</t>
+          <t>COALESCE(nome, ID).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_deals_stage</t>
+          <t>vw_hubspot_contacts_lifecycle</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Deal_Created_Date / Deal_Closed_Date</t>
+          <t>Became_Lead/MQL/SQL/Opportunity/Customer_Date</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2016,7 +2017,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Criação / fechamento (real só quando fechado).</t>
+          <t>Data de entrada em cada estágio (modelo v2).</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2029,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Origem</t>
+          <t>Deal_ID</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -2038,7 +2039,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Herdada do contato associado.</t>
+          <t>Chave do negócio.</t>
         </is>
       </c>
     </row>
@@ -2050,17 +2051,17 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Campaign_ID / Campanha</t>
+          <t>Deal_Status / Deal_Win</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>STRING</t>
+          <t>STRING/BOOL</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Campanha (via contato).</t>
+          <t>open|won|lost / ganho.</t>
         </is>
       </c>
     </row>
@@ -2072,103 +2073,191 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Contact_ID</t>
+          <t>Deal_Amount / Deal_Currency</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
+          <t>NUMERIC/STRING</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Valor e moeda (BRL).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>vw_hubspot_deals_stage</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Deal_Created_Date / Deal_Closed_Date</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Criação / fechamento (real só quando fechado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>vw_hubspot_deals_stage</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
           <t>STRING</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Contato associado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>vw_hubspot_stage_events</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>entity_id</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>ID do contato ou deal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>vw_hubspot_stage_events</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>stage</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>contact_created|lead|mql|sql|opportunity|client|deal_created|deal_won|deal_lost.</t>
+          <t>Herdada do contato associado.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>vw_hubspot_stage_events</t>
+          <t>vw_hubspot_deals_stage</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>event_date</t>
+          <t>Campaign_ID / Campanha</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>STRING</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Data em que o estágio ocorreu.</t>
+          <t>Campanha (via contato).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
+          <t>vw_hubspot_deals_stage</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Contact_ID</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>STRING</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Contato associado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
           <t>vw_hubspot_stage_events</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>entity_id</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>STRING</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>ID do contato ou deal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>vw_hubspot_stage_events</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>STRING</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>contact_created|lead|mql|sql|opportunity|client|deal_created|deal_won|deal_lost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>vw_hubspot_stage_events</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>event_date</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Data em que o estágio ocorreu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>vw_hubspot_stage_events</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>origem / campanha / campaign_id</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>STRING</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>Dimensões carregadas para a agregação.</t>
         </is>
@@ -3206,4 +3295,195 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002E7D52"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="74" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Estado real &amp; correções (jul/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Validação da revisão técnica após o deploy no n8n. Volume real, correções aplicadas e pendências fora do BigQuery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Situação</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Detalhe / ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Volume carregado</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>~18.682 contacts e 17.046 deals no clean (backfill rodou). Deals amount total na base: R$ 7,26 bi (todos) / R$ 639,3 mi (ganhos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>amount = 0 na view de funil</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>CORRIGIDO</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Era LEFT JOIN por 'campanha' NULL (deals Offline). Agora o amount é somado no próprio fato (evento deal_won). Validado: R$ 639,3 mi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Meio do funil (MQL/SQL/Opp)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>ESCLARECIDO</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>MQL popula (1.816). SQL (15) e Opportunity (6) ~0 porque a conta NÃO usa esses estágios de lifecycle (vai Lead→MQL→Cliente). Mapeamento hs_v2_* correto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Deals sem contato associado</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>DADO DE ORIGEM</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>98% dos deals NÃO têm contato associado no próprio HubSpot (o import não vinculou). A captura no n8n está certa (associations vem em 100% dos payloads, mas vazio). Correção: associar no HubSpot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Acesso da SA à consolidada</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>PENDENTE (fora do BQ)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>dataViewer no dataset cobre as tabelas HubSpot (nativas). A vw_ads_crm_results lê RD/Hotmart que são janelas para Google Sheets → precisa COMPARTILHAR as planilhas com a SA no Google Drive. Enquanto isso, dashboard lê vw_hubspot_leads_stages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Join de campanha — Google</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Paid Search: HubSpot grava o ID da campanha → bate com as tabelas de Ads por Campaign_ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="75" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Join de campanha — Meta</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>PENDENTE (fora do BQ)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Meta não expõe ID no HubSpot (só nome). Nomes divergem (caixa / automáticos). Correção na origem: conectar Meta Ads no HubSpot (passa a gravar ID) OU padronizar nomes das campanhas no Meta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Multi-cliente</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>ATENÇÃO</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>vw_ads_crm_results tem VÁRIOS clientes (account_id/account_name). O dashboard TEM que filtrar por conta. As vw_hubspot_* são só HubSpot.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>